<commit_message>
Q19 refine: add ROI context, option 1 ASAP
</commit_message>
<xml_diff>
--- a/AutomateX_Scorecard_Ground_Truth.xlsx
+++ b/AutomateX_Scorecard_Ground_Truth.xlsx
@@ -2096,12 +2096,12 @@
       </c>
       <c r="D23" s="31" t="inlineStr">
         <is>
-          <t>If we identified a clear, costed automation opportunity that fit your team, how soon would you be open to a paid pilot to prove it out?</t>
+          <t>If we identified a clear automation opportunity that fits your team and with demonstrated return on investment, how soon would you be open to a paid pilot to prove it out?</t>
         </is>
       </c>
       <c r="E23" s="31" t="inlineStr">
         <is>
-          <t>Yes, within the next 30 days if the fit is right.</t>
+          <t>Yes, and ASAP.</t>
         </is>
       </c>
       <c r="F23" s="31" t="inlineStr">

</xml_diff>

<commit_message>
Band ladder descriptions: short one-line meaning per maturity band + hover tooltips
</commit_message>
<xml_diff>
--- a/AutomateX_Scorecard_Ground_Truth.xlsx
+++ b/AutomateX_Scorecard_Ground_Truth.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -160,8 +160,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -216,6 +222,11 @@
         <bgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1F36"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -251,7 +262,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -396,6 +407,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3336,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="25" min="1" max="1"/>
@@ -3344,6 +3361,7 @@
     <col width="36" customWidth="1" style="25" min="4" max="4"/>
     <col width="16" customWidth="1" style="25" min="5" max="5"/>
     <col width="36" customWidth="1" style="25" min="6" max="6"/>
+    <col width="48" customWidth="1" style="26" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" s="26">
@@ -3651,6 +3669,11 @@
         </is>
       </c>
       <c r="F14" s="29" t="n"/>
+      <c r="G14" s="49" t="inlineStr">
+        <is>
+          <t>Viewer description (shown under band ladder)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="31.5" customHeight="1" s="26">
       <c r="A15" s="31" t="inlineStr">
@@ -3679,6 +3702,11 @@
         </is>
       </c>
       <c r="F15" s="31" t="n"/>
+      <c r="G15" s="50" t="inlineStr">
+        <is>
+          <t>Each project starts from scratch. Heroes carry the firm.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="31.5" customHeight="1" s="26">
       <c r="A16" s="31" t="inlineStr">
@@ -3707,6 +3735,11 @@
         </is>
       </c>
       <c r="F16" s="31" t="n"/>
+      <c r="G16" s="50" t="inlineStr">
+        <is>
+          <t>Foundations exist. Lessons captured, but compounding is inconsistent.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="31.5" customHeight="1" s="26">
       <c r="A17" s="31" t="inlineStr">
@@ -3735,6 +3768,11 @@
         </is>
       </c>
       <c r="F17" s="31" t="n"/>
+      <c r="G17" s="50" t="inlineStr">
+        <is>
+          <t>The mechanics work. Specific friction points limit further gains.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="31.5" customHeight="1" s="26">
       <c r="A18" s="31" t="inlineStr">
@@ -3763,6 +3801,11 @@
         </is>
       </c>
       <c r="F18" s="31" t="n"/>
+      <c r="G18" s="50" t="inlineStr">
+        <is>
+          <t>Runs on a system that compounds. AI is evidenceable, not aspirational.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>